<commit_message>
Removing extra sheet from results xlsx file
</commit_message>
<xml_diff>
--- a/results/results_iter1.xlsx
+++ b/results/results_iter1.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danemerson/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danemerson/Documents/CMU/01_Research/Projects/CPA/Bayesian Optimization/cpa-bayesian-opt/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71B0E3D-783B-AB4C-83F0-211B7C863661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97DDB7E7-8896-2147-A90E-DDAC7115A8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="36900" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35840" windowHeight="19780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Duplicates" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>Index</t>
   </si>
@@ -196,9 +195,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>SD(wthin experimental values =3)</t>
   </si>
   <si>
     <t>Predicted - experimental</t>
@@ -668,16 +664,16 @@
         <v>52</v>
       </c>
       <c r="O1" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="P1" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="Q1" s="2" t="s">
         <v>53</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
@@ -2803,551 +2799,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C55DF65-E6B8-234F-B772-91D04E30071C}">
-  <dimension ref="A1:R14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>6</v>
-      </c>
-      <c r="J3" s="3">
-        <v>67.279710489764682</v>
-      </c>
-      <c r="L3">
-        <v>63.018521353130268</v>
-      </c>
-      <c r="M3">
-        <v>66.719033977143212</v>
-      </c>
-      <c r="N3">
-        <v>68.63938053097344</v>
-      </c>
-      <c r="O3" s="3">
-        <f t="shared" ref="O3:O5" si="0">AVERAGE(L3:N3)</f>
-        <v>66.125645287082307</v>
-      </c>
-      <c r="P3">
-        <f t="shared" ref="P3:P5" si="1">_xlfn.STDEV.P(L3:N3)</f>
-        <v>2.3327518909941398</v>
-      </c>
-      <c r="R3">
-        <f t="shared" ref="R3:R5" si="2">J3-O3</f>
-        <v>1.154065202682375</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>6</v>
-      </c>
-      <c r="J4" s="3">
-        <v>67.279710489764696</v>
-      </c>
-      <c r="L4">
-        <v>64.549211694474209</v>
-      </c>
-      <c r="M4">
-        <v>62.726796660813847</v>
-      </c>
-      <c r="N4">
-        <v>63.329646017699105</v>
-      </c>
-      <c r="O4" s="3">
-        <f t="shared" si="0"/>
-        <v>63.535218124329049</v>
-      </c>
-      <c r="P4">
-        <f t="shared" si="1"/>
-        <v>0.75806510582140707</v>
-      </c>
-      <c r="R4">
-        <f t="shared" si="2"/>
-        <v>3.7444923654356472</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>6</v>
-      </c>
-      <c r="J5" s="3">
-        <v>67.272590659985426</v>
-      </c>
-      <c r="L5">
-        <v>62.651155671207718</v>
-      </c>
-      <c r="M5">
-        <v>55.518590395219164</v>
-      </c>
-      <c r="N5">
-        <v>51.935840707964587</v>
-      </c>
-      <c r="O5" s="3">
-        <f t="shared" si="0"/>
-        <v>56.70186225813049</v>
-      </c>
-      <c r="P5">
-        <f t="shared" si="1"/>
-        <v>4.4538068298586824</v>
-      </c>
-      <c r="R5">
-        <f t="shared" si="2"/>
-        <v>10.570728401854936</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>1.5</v>
-      </c>
-      <c r="F7">
-        <v>0.5</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7" s="3">
-        <v>103.704895489573</v>
-      </c>
-      <c r="L7">
-        <v>94.734425225776832</v>
-      </c>
-      <c r="M7">
-        <v>92.335890090256598</v>
-      </c>
-      <c r="N7">
-        <v>92.865044247787594</v>
-      </c>
-      <c r="O7" s="3">
-        <f t="shared" ref="O7:O8" si="3">AVERAGE(L7:N7)</f>
-        <v>93.311786521273675</v>
-      </c>
-      <c r="P7">
-        <f t="shared" ref="P7:P8" si="4">_xlfn.STDEV.P(L7:N7)</f>
-        <v>1.0288915372933796</v>
-      </c>
-      <c r="R7">
-        <f t="shared" ref="R7:R8" si="5">J7-O7</f>
-        <v>10.39310896829933</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>1.5</v>
-      </c>
-      <c r="F8">
-        <v>0.5</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>2</v>
-      </c>
-      <c r="J8" s="3">
-        <v>104.199949060631</v>
-      </c>
-      <c r="L8">
-        <v>97.857033522118471</v>
-      </c>
-      <c r="M8">
-        <v>96.383575147090525</v>
-      </c>
-      <c r="N8">
-        <v>88.938053097345104</v>
-      </c>
-      <c r="O8" s="3">
-        <f t="shared" si="3"/>
-        <v>94.392887255518033</v>
-      </c>
-      <c r="P8">
-        <f t="shared" si="4"/>
-        <v>3.903774384328806</v>
-      </c>
-      <c r="R8">
-        <f t="shared" si="5"/>
-        <v>9.8070618051129657</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10">
-        <v>3</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>0.5</v>
-      </c>
-      <c r="F10">
-        <v>0.5</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>5</v>
-      </c>
-      <c r="J10" s="3">
-        <v>87.231381736608142</v>
-      </c>
-      <c r="L10">
-        <v>84.876779427521825</v>
-      </c>
-      <c r="M10">
-        <v>82.410744539937781</v>
-      </c>
-      <c r="N10">
-        <v>78.429203539822993</v>
-      </c>
-      <c r="O10" s="3">
-        <f t="shared" ref="O10:O11" si="6">AVERAGE(L10:N10)</f>
-        <v>81.905575835760871</v>
-      </c>
-      <c r="P10">
-        <f t="shared" ref="P10:P11" si="7">_xlfn.STDEV.P(L10:N10)</f>
-        <v>2.6563389933852797</v>
-      </c>
-      <c r="R10">
-        <f t="shared" ref="R10:R11" si="8">J10-O10</f>
-        <v>5.3258059008472713</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11">
-        <v>3</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>0.5</v>
-      </c>
-      <c r="F11">
-        <v>0.5</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
-        <v>5</v>
-      </c>
-      <c r="J11" s="3">
-        <v>88.675724977200744</v>
-      </c>
-      <c r="L11">
-        <v>76.366141129649478</v>
-      </c>
-      <c r="M11">
-        <v>84.351415457597867</v>
-      </c>
-      <c r="N11">
-        <v>77.212389380530965</v>
-      </c>
-      <c r="O11" s="3">
-        <f t="shared" si="6"/>
-        <v>79.309981989259441</v>
-      </c>
-      <c r="P11">
-        <f t="shared" si="7"/>
-        <v>3.5815334320457519</v>
-      </c>
-      <c r="R11">
-        <f t="shared" si="8"/>
-        <v>9.365742987941303</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13">
-        <v>2.5</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0.5</v>
-      </c>
-      <c r="E13">
-        <v>0.5</v>
-      </c>
-      <c r="F13">
-        <v>0.5</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <v>4</v>
-      </c>
-      <c r="J13" s="3">
-        <v>98.069933531006626</v>
-      </c>
-      <c r="L13">
-        <v>93.816011020970464</v>
-      </c>
-      <c r="M13">
-        <v>86.458429596771708</v>
-      </c>
-      <c r="N13">
-        <v>83.019911504424769</v>
-      </c>
-      <c r="O13" s="3">
-        <f t="shared" ref="O13:O14" si="9">AVERAGE(L13:N13)</f>
-        <v>87.764784040722319</v>
-      </c>
-      <c r="P13">
-        <f t="shared" ref="P13:P14" si="10">_xlfn.STDEV.P(L13:N13)</f>
-        <v>4.5032479125413225</v>
-      </c>
-      <c r="R13">
-        <f t="shared" ref="R13:R14" si="11">J13-O13</f>
-        <v>10.305149490284307</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14">
-        <v>2.5</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>0.5</v>
-      </c>
-      <c r="E14">
-        <v>0.5</v>
-      </c>
-      <c r="F14">
-        <v>0.5</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>4</v>
-      </c>
-      <c r="J14" s="3">
-        <v>99.431369332052782</v>
-      </c>
-      <c r="L14">
-        <v>90.509719883667529</v>
-      </c>
-      <c r="M14">
-        <v>88.066414071404353</v>
-      </c>
-      <c r="N14">
-        <v>75.663716814159272</v>
-      </c>
-      <c r="O14" s="3">
-        <f t="shared" si="9"/>
-        <v>84.746616923077056</v>
-      </c>
-      <c r="P14">
-        <f t="shared" si="10"/>
-        <v>6.4995764792532809</v>
-      </c>
-      <c r="R14">
-        <f t="shared" si="11"/>
-        <v>14.684752408975726</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>